<commit_message>
Pollos: calculadora Excel con la parte 2 (capacidad, galpón, presupuesto, equilibrio, flujo y escenarios)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/materiales/calculadora-lote-pollos-engorde.xlsx
+++ b/materiales/calculadora-lote-pollos-engorde.xlsx
@@ -6,13 +6,16 @@
   <sheets>
     <sheet sheetId="1" name="Instrucciones" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Calculadora" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Capacidad y galpón" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Presupuesto y equilibrio" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Escenarios" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="120">
   <si>
     <t>Calculadora básica del lote · Pollos de engorde</t>
   </si>
@@ -47,6 +50,21 @@
     <t>costo por kg = costo total ÷ kg vendidos · ingreso = kg vendidos × precio · beneficio = ingreso − costo total · margen = beneficio ÷ ingreso</t>
   </si>
   <si>
+    <t>PARTE 2 · SU PROYECTO (módulos 9 a 12)</t>
+  </si>
+  <si>
+    <t>• «Capacidad y galpón»: lotes por año, pollos y kilos al año, área y largo del galpón, comederos, bebederos y niples (módulos 9 y 10).</t>
+  </si>
+  <si>
+    <t>• «Presupuesto y equilibrio»: inversión inicial, precio y kilos de equilibrio, capital de trabajo, lotes y años para recuperar la inversión, y el flujo de caja semana a semana (módulo 11).</t>
+  </si>
+  <si>
+    <t>• «Escenarios»: beneficio del lote con tres mortalidades y tres precios, en rojo, amarillo o verde (módulo 11).</t>
+  </si>
+  <si>
+    <t>Todos los importes de ejemplo son ILUSTRATIVOS y no garantizan ganancias: use sus cotizaciones, sus costos y el precio que le ofrezcan sus compradores.</t>
+  </si>
+  <si>
     <t>Calculadora básica del lote</t>
   </si>
   <si>
@@ -120,20 +138,259 @@
   </si>
   <si>
     <t>Conversión alimenticia</t>
+  </si>
+  <si>
+    <t>Capacidad anual y tamaño del galpón</t>
+  </si>
+  <si>
+    <t>Amarillo = se escribe (trae un EJEMPLO ILUSTRATIVO: sustitúyalo por sus datos) · Gris = se calcula solo</t>
+  </si>
+  <si>
+    <t>Datos (módulos 9 y 10)</t>
+  </si>
+  <si>
+    <t>Pollitos por lote</t>
+  </si>
+  <si>
+    <t>Semanas de crianza</t>
+  </si>
+  <si>
+    <t>Semanas de vacío sanitario</t>
+  </si>
+  <si>
+    <t>No lo recorte: protege al lote siguiente</t>
+  </si>
+  <si>
+    <t>Mortalidad prevista (%)</t>
+  </si>
+  <si>
+    <t>Peso de venta (kg)</t>
+  </si>
+  <si>
+    <t>Densidad (pollos/m²)</t>
+  </si>
+  <si>
+    <t>Más de 12 es alto para galpón abierto en clima cálido</t>
+  </si>
+  <si>
+    <t>Ancho del galpón (m)</t>
+  </si>
+  <si>
+    <t>Pollos por comedero de tolva</t>
+  </si>
+  <si>
+    <t>Pollos por bebedero de campana</t>
+  </si>
+  <si>
+    <t>Pollos por niple</t>
+  </si>
+  <si>
+    <t>Semanas por ciclo</t>
+  </si>
+  <si>
+    <t>Lotes por año (exacto)</t>
+  </si>
+  <si>
+    <t>52 semanas ÷ ciclo</t>
+  </si>
+  <si>
+    <t>Lotes para planificar</t>
+  </si>
+  <si>
+    <t>redondeado hacia abajo</t>
+  </si>
+  <si>
+    <t>Pollitos al año</t>
+  </si>
+  <si>
+    <t>Pollos vendidos al año</t>
+  </si>
+  <si>
+    <t>Kg vendidos al año</t>
+  </si>
+  <si>
+    <t>Área de piso (m²)</t>
+  </si>
+  <si>
+    <t>Largo del galpón (m)</t>
+  </si>
+  <si>
+    <t>Comederos de tolva</t>
+  </si>
+  <si>
+    <t>hacia arriba</t>
+  </si>
+  <si>
+    <t>Bebederos de campana</t>
+  </si>
+  <si>
+    <t>o bien niples</t>
+  </si>
+  <si>
+    <t>Medidas y capacidades orientativas: confírmelas con su técnico, la guía de su línea y el fabricante del equipo.</t>
+  </si>
+  <si>
+    <t>Presupuesto, punto de equilibrio y flujo de caja</t>
+  </si>
+  <si>
+    <t>Inversión inicial (pida 2 cotizaciones por renglón)</t>
+  </si>
+  <si>
+    <t>Galpón de 100 m²: estructura, techo y piso</t>
+  </si>
+  <si>
+    <t>Malla, cortinas y puertas</t>
+  </si>
+  <si>
+    <t>Comederos, bebederos, criadoras, balanza y termómetros</t>
+  </si>
+  <si>
+    <t>Tanque, tubería y filtro de agua</t>
+  </si>
+  <si>
+    <t>Instalación eléctrica y bombillos</t>
+  </si>
+  <si>
+    <t>Bodega, pediluvio y cerca perimetral</t>
+  </si>
+  <si>
+    <t>Inversión inicial total</t>
+  </si>
+  <si>
+    <t>Datos de un lote</t>
+  </si>
+  <si>
+    <t>Costo total del lote (RD$)</t>
+  </si>
+  <si>
+    <t>Use la hoja «Calculadora»</t>
+  </si>
+  <si>
+    <t>De eso, depreciación (RD$)</t>
+  </si>
+  <si>
+    <t>Desgaste del galpón y del equipo</t>
+  </si>
+  <si>
+    <t>Pollitos del lote</t>
+  </si>
+  <si>
+    <t>Lotes al año</t>
+  </si>
+  <si>
+    <t>Hoja «Capacidad y galpón»</t>
+  </si>
+  <si>
+    <t>Reserva sobre el capital de trabajo (%)</t>
+  </si>
+  <si>
+    <t>Precio de equilibrio (RD$/kg)</t>
+  </si>
+  <si>
+    <t>Por debajo de este precio, el lote pierde</t>
+  </si>
+  <si>
+    <t>Kg de equilibrio a su precio</t>
+  </si>
+  <si>
+    <t>Ingreso del lote</t>
+  </si>
+  <si>
+    <t>Beneficio del lote</t>
+  </si>
+  <si>
+    <t>Capital de trabajo</t>
+  </si>
+  <si>
+    <t>(costo − depreciación) × (1 + reserva)</t>
+  </si>
+  <si>
+    <t>Caja que deja cada lote</t>
+  </si>
+  <si>
+    <t>beneficio + depreciación</t>
+  </si>
+  <si>
+    <t>Lotes para recuperar la inversión</t>
+  </si>
+  <si>
+    <t>Años aproximados</t>
+  </si>
+  <si>
+    <t>Flujo de caja de un lote (salidas de efectivo por semana)</t>
+  </si>
+  <si>
+    <t>Sale (RD$)</t>
+  </si>
+  <si>
+    <t>Saldo acumulado</t>
+  </si>
+  <si>
+    <t>Semana 0 (pollitos, cama y preparación)</t>
+  </si>
+  <si>
+    <t>Semana 1</t>
+  </si>
+  <si>
+    <t>Semana 2</t>
+  </si>
+  <si>
+    <t>Semana 3</t>
+  </si>
+  <si>
+    <t>Semana 4</t>
+  </si>
+  <si>
+    <t>Semana 5</t>
+  </si>
+  <si>
+    <t>Semana 6</t>
+  </si>
+  <si>
+    <t>Venta (entra el ingreso del lote)</t>
+  </si>
+  <si>
+    <t>Punto más bajo del saldo</t>
+  </si>
+  <si>
+    <t>Es el dinero mínimo que debe tener antes de empezar</t>
+  </si>
+  <si>
+    <t>Si el comprador paga a 15 días, el punto bajo dura dos semanas más. EJEMPLO ILUSTRATIVO: no garantiza ganancias.</t>
+  </si>
+  <si>
+    <t>¿Y si las cosas no salen como espero?</t>
+  </si>
+  <si>
+    <t>Mortalidad ↓ · Precio RD$/kg →</t>
+  </si>
+  <si>
+    <t>Beneficio del lote (RD$)</t>
+  </si>
+  <si>
+    <t>Escriba sus mortalidades y precios</t>
+  </si>
+  <si>
+    <t>Rojo = pierde · Amarillo = gana poco (menos de RD$ 15,000) · Verde = gana. Mire siempre la esquina de abajo a la izquierda.</t>
+  </si>
+  <si>
+    <t>Beneficio = pollos vivos × peso × precio − costo. EJEMPLO ILUSTRATIVO: sustituya por los costos y precios reales de su granja.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="&quot;RD$&quot; #,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="&quot;RD$&quot; #,##0"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
+    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="&quot;+RD$&quot; #,##0;&quot;−RD$&quot; #,##0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -153,6 +410,11 @@
     <font>
       <b/>
       <color rgb="FF7C2D12"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF7C2D12"/>
       <sz val="16"/>
     </font>
     <font>
@@ -163,6 +425,9 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="5">
@@ -215,7 +480,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -226,9 +491,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
@@ -255,11 +523,87 @@
     <xf numFmtId="168" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="right"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="10">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC4544A"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4D3D0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF6E7C1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD3EADB"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -604,7 +948,7 @@
   <sheetPr>
     <tabColor rgb="FFC2410C"/>
   </sheetPr>
-  <dimension ref="B1:B12"/>
+  <dimension ref="B1:B18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -669,6 +1013,36 @@
     <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -692,182 +1066,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>11</v>
+      <c r="A1" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>12</v>
+      <c r="A2" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="6"/>
+      <c r="A4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="7"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="8">
+      <c r="A5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="9">
         <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="9">
+      <c r="A6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="10">
         <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="8">
+      <c r="A7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="9">
         <v>2000</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="9">
+      <c r="A8" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="10">
         <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="10">
+      <c r="A9" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="11">
         <v>0.04</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>19</v>
+      <c r="C9" s="12" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="12">
+      <c r="A10" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="13">
         <v>2.3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="13">
+      <c r="A11" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="14">
         <v>0.04</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="9">
+      <c r="A12" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="10">
         <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="14">
+      <c r="A13" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="15">
         <v>22000</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="6"/>
+      <c r="A15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="7"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="15">
+      <c r="A16" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="16">
         <f>IF(B5="","falta dato",ROUND(B5*(1-IF(B9="",0,B9)),0))</f>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="B17" s="16">
+      <c r="A17" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="17">
         <f>IF(OR(B5="",B6="",B7="",B8=""),"falta dato",B5*B6+B7*B8+IF(B13="",0,B13))</f>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="17">
+      <c r="A18" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" s="18">
         <f>IF(OR(NOT(ISNUMBER(B16)),NOT(ISNUMBER(B17))),"falta dato",IF(B16&lt;=0,"falta dato",B17/B16))</f>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="18">
+      <c r="A19" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="19">
         <f>IF(OR(NOT(ISNUMBER(B16)),B10=""),"falta dato",B16*B10)</f>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B20" s="18">
+      <c r="A20" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="19">
         <f>IF(OR(NOT(ISNUMBER(B19)),B5="",B11=""),"falta dato",B19-B5*B11)</f>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="17">
+      <c r="A21" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="18">
         <f>IF(OR(NOT(ISNUMBER(B17)),NOT(ISNUMBER(B19))),"falta dato",IF(B19&lt;=0,"falta dato",B17/B19))</f>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>31</v>
+      <c r="C21" s="12" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="16">
+      <c r="A22" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="17">
         <f>IF(OR(NOT(ISNUMBER(B19)),B12=""),"falta dato",B19*B12)</f>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="16">
+      <c r="A23" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="17">
         <f>IF(OR(NOT(ISNUMBER(B22)),NOT(ISNUMBER(B17))),"falta dato",B22-B17)</f>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="19">
+      <c r="A24" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="20">
         <f>IF(NOT(ISNUMBER(B23)),"falta dato",IF(B22&lt;=0,"falta dato",B23/B22))</f>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B25" s="20">
+      <c r="A25" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="21">
         <f>IF(OR(B7="",NOT(ISNUMBER(B20))),"falta dato",IF(B20&lt;=0,"falta dato",B7/B20))</f>
       </c>
     </row>
@@ -890,4 +1264,821 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF1F6F8B"/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="7"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="22">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="22">
+        <v>2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="11">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="13">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="23">
+        <v>10</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="23">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="22">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" s="22">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="22">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="7"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="24">
+        <f>IF(OR(B6="",B7=""),"falta dato",IFERROR(B6+B7,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" s="25">
+        <f>IF(OR(B17=""),"falta dato",IFERROR(52/B17,"falta dato"))</f>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B19" s="24">
+        <f>IF(OR(B18=""),"falta dato",IFERROR(ROUNDDOWN(B18,0),"falta dato"))</f>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="16">
+        <f>IF(OR(B5="",B19=""),"falta dato",IFERROR(B5*B19,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="16">
+        <f>IF(OR(B5="",B19=""),"falta dato",IFERROR(ROUND(B5*(1-B8),0)*B19,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="16">
+        <f>IF(OR(B21="",B9=""),"falta dato",IFERROR(B21*B9,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="19">
+        <f>IF(OR(B5="",B10=""),"falta dato",IFERROR(B5/B10,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="19">
+        <f>IF(OR(B23="",B11=""),"falta dato",IFERROR(B23/B11,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="16">
+        <f>IF(OR(B5="",B12=""),"falta dato",IFERROR(ROUNDUP(B5/B12,0),"falta dato"))</f>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" s="16">
+        <f>IF(OR(B5="",B13=""),"falta dato",IFERROR(ROUNDUP(B5/B13,0),"falta dato"))</f>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B27" s="16">
+        <f>IF(OR(B5="",B14=""),"falta dato",IFERROR(ROUNDUP(B5/B14,0),"falta dato"))</f>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0"/>
+  <conditionalFormatting sqref="B17:B27">
+    <cfRule type="containsText" dxfId="9" priority="1">
+      <formula>NOT(ISERROR(SEARCH("falta",B17)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Número" error="No puede ser negativo." sqref="B5:B14">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Mortalidad" error="Escriba un porcentaje entre 0 % y 100 %." sqref="B8">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF9A6D14"/>
+  </sheetPr>
+  <dimension ref="A1:C47"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="7"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" s="15">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" s="15">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="15">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="15">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="15">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="15">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B11" s="17">
+        <f>SUM(B5:B10)</f>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B13" s="7"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="15">
+        <v>240000</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="15">
+        <v>4000</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="11">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="13">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="10">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="22">
+        <v>6</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="B21" s="11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="7"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="16">
+        <f>IF(OR(B16=""),"falta dato",IFERROR(ROUND(B16*(1-B17),0),"falta dato"))</f>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="19">
+        <f>IF(OR(B24="",B18=""),"falta dato",IFERROR(B24*B18,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B26" s="18">
+        <f>IF(OR(B14="",B25=""),"falta dato",IFERROR(B14/B25,"falta dato"))</f>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B27" s="16">
+        <f>IF(OR(B14="",B19=""),"falta dato",IFERROR(B14/B19,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="17">
+        <f>IF(OR(B25="",B19=""),"falta dato",IFERROR(B25*B19,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" s="17">
+        <f>IF(OR(B28="",B14=""),"falta dato",IFERROR(B28-B14,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" s="17">
+        <f>IF(OR(B14=""),"falta dato",IFERROR((B14-B15)*(1+B21),"falta dato"))</f>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" s="17">
+        <f>IF(OR(B29=""),"falta dato",IFERROR(B29+B15,"falta dato"))</f>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B32" s="25">
+        <f>IF(OR(B31=""),"falta dato",IFERROR(IF(B31&lt;=0,"no se recupera",B11/B31),"falta dato"))</f>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B33" s="25">
+        <f>IF(OR(B32="",B20=""),"falta dato",IFERROR(IF(ISNUMBER(B32),B32/B20,"no se recupera"),"falta dato"))</f>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="26" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B37" s="15">
+        <v>72000</v>
+      </c>
+      <c r="C37" s="27">
+        <f>-B37</f>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B38" s="15">
+        <v>10000</v>
+      </c>
+      <c r="C38" s="27">
+        <f>C37-B38</f>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="B39" s="15">
+        <v>17000</v>
+      </c>
+      <c r="C39" s="27">
+        <f>C38-B39</f>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B40" s="15">
+        <v>27000</v>
+      </c>
+      <c r="C40" s="27">
+        <f>C39-B40</f>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="B41" s="15">
+        <v>38000</v>
+      </c>
+      <c r="C41" s="27">
+        <f>C40-B41</f>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="B42" s="15">
+        <v>44000</v>
+      </c>
+      <c r="C42" s="27">
+        <f>C41-B42</f>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" s="15">
+        <v>28000</v>
+      </c>
+      <c r="C43" s="27">
+        <f>C42-B43</f>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B44" s="27">
+        <f>IF(ISNUMBER(B28),B28,0)</f>
+      </c>
+      <c r="C44" s="27">
+        <f>C43+B44</f>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="B45" s="17">
+        <f>MIN(C37:C43)</f>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="12" t="s">
+        <v>113</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0"/>
+  <conditionalFormatting sqref="B24:B33">
+    <cfRule type="containsText" dxfId="9" priority="1">
+      <formula>NOT(ISERROR(SEARCH("falta",B24)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="1">
+      <formula>NOT(ISERROR(SEARCH("no se recupera",B24)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B29">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C37:C44">
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Número" error="No puede ser negativo." sqref="B37:B43">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Número" error="No puede ser negativo." sqref="B5:B21">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FFB42318"/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="46" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="7"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="13">
+        <v>2.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B7" s="15">
+        <v>240000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" s="28">
+        <v>105</v>
+      </c>
+      <c r="C10" s="28">
+        <v>115</v>
+      </c>
+      <c r="D10" s="28">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="29">
+        <v>0.03</v>
+      </c>
+      <c r="B11" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A11="",B$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A11),0)*$B$6*B$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="C11" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A11="",C$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A11),0)*$B$6*C$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="D11" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A11="",D$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A11),0)*$B$6*D$10-$B$7,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="29">
+        <v>0.06</v>
+      </c>
+      <c r="B12" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A12="",B$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A12),0)*$B$6*B$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="C12" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A12="",C$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A12),0)*$B$6*C$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="D12" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A12="",D$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A12),0)*$B$6*D$10-$B$7,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="29">
+        <v>0.1</v>
+      </c>
+      <c r="B13" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A13="",B$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A13),0)*$B$6*B$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="C13" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A13="",C$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A13),0)*$B$6*C$10-$B$7,"falta dato"))</f>
+      </c>
+      <c r="D13" s="30">
+        <f>IF(OR($B$5="",$B$6="",$B$7="",$A13="",D$10=""),"falta dato",IFERROR(ROUND($B$5*(1-$A13),0)*$B$6*D$10-$B$7,"falta dato"))</f>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection sheet="1" formatColumns="0" formatRows="0"/>
+  <conditionalFormatting sqref="B11:D13">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="between">
+      <formula>0</formula>
+      <formula>14999.99</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="3" operator="greaterThanOrEqual">
+      <formula>15000</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="1">
+      <formula>NOT(ISERROR(SEARCH("falta",B11)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Número" error="No puede ser negativo." sqref="B5:B7">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>